<commit_message>
Traduction des libellés de Composition.section 1fb7579c178fac8b0a8f36cc8b385ec2a9b08bf8
</commit_message>
<xml_diff>
--- a/composition-eu-parent/ig/StructureDefinition-fr-composition-document.xlsx
+++ b/composition-eu-parent/ig/StructureDefinition-fr-composition-document.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9227" uniqueCount="892">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9227" uniqueCount="893">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-02T12:41:40+00:00</t>
+    <t>2026-10-02T12:54:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2549,7 +2549,7 @@
     <t>Composition.section</t>
   </si>
   <si>
-    <t>Composition is broken into sections</t>
+    <t>Section</t>
   </si>
   <si>
     <t>The root of the sections that make up the composition.</t>
@@ -2568,6 +2568,9 @@
     <t>Composition.section.id</t>
   </si>
   <si>
+    <t>Identifiant technique</t>
+  </si>
+  <si>
     <t>Composition.section.extension</t>
   </si>
   <si>
@@ -2581,7 +2584,7 @@
 </t>
   </si>
   <si>
-    <t>Commentaires supplémentaires pour chaque section.</t>
+    <t>Commentaires.</t>
   </si>
   <si>
     <t>Permet de porter des commentaires dans chaque section.</t>
@@ -2600,7 +2603,7 @@
 labelcaption</t>
   </si>
   <si>
-    <t>Label for section (e.g. for ToC)</t>
+    <t>Titre de la section</t>
   </si>
   <si>
     <t>The label for this particular section.  This will be part of the rendered content for the document, and is often used to build a table of contents.</t>
@@ -2615,7 +2618,7 @@
     <t>Composition.section.code</t>
   </si>
   <si>
-    <t>Classification of section (recommended)</t>
+    <t>Code de la section</t>
   </si>
   <si>
     <t>A code identifying the kind of content contained within the section. This must be consistent with the section title.</t>
@@ -2638,7 +2641,7 @@
 </t>
   </si>
   <si>
-    <t>Who and/or what authored the section</t>
+    <t>Auteur de la section</t>
   </si>
   <si>
     <t>Identifies who is responsible for the information in this section, not necessarily who typed it in.</t>
@@ -2647,7 +2650,7 @@
     <t>Composition.section.focus</t>
   </si>
   <si>
-    <t>Who/what the section is about, when it is not about the subject of composition</t>
+    <t>Sujet de la section (si différent du sujet de la composition)</t>
   </si>
   <si>
     <t>The actual focus of the section when it is not the subject of the composition, but instead represents something or someone associated with the subject such as (for a patient subject) a spouse, parent, fetus, or donor. If not focus is specified, the focus is assumed to be focus of the parent section, or, for a section in the Composition itself, the subject of the composition. Sections with a focus SHALL only include resources where the logical subject (patient, subject, focus, etc.) matches the section focus, or the resources have no logical subject (few resources).</t>
@@ -2662,7 +2665,7 @@
     <t>Composition.section.text</t>
   </si>
   <si>
-    <t>Text summary of the section, for human interpretation</t>
+    <t>Partie narrative de la section (pour affichage à un humain)</t>
   </si>
   <si>
     <t>A human-readable narrative that contains the attested content of the section, used to represent the content of the resource to a human. The narrative need not encode all the structured data, but is required to contain sufficient detail to make it "clinically safe" for a human to just read the narrative.</t>
@@ -2681,7 +2684,7 @@
     <t>Composition.section.mode</t>
   </si>
   <si>
-    <t>working | snapshot | changes</t>
+    <t>Type de section (Liste de référence, Liste à date, Liste des modifications)</t>
   </si>
   <si>
     <t>How the entry list was prepared - whether it is a working list that is suitable for being maintained on an ongoing basis, or if it represents a snapshot of a list of items from another source, or whether it is a prepared list where items may be marked as added, modified or deleted.</t>
@@ -2705,7 +2708,7 @@
     <t>Composition.section.orderedBy</t>
   </si>
   <si>
-    <t>Order of section entries</t>
+    <t>Ordre des entrées</t>
   </si>
   <si>
     <t>Specifies the order applied to the items in the section entries.</t>
@@ -2729,7 +2732,7 @@
     <t>Composition.section.entry</t>
   </si>
   <si>
-    <t>A reference to data that supports this section</t>
+    <t>Entrée</t>
   </si>
   <si>
     <t>A reference to the actual resource from which the narrative in the section is derived.</t>
@@ -2751,7 +2754,7 @@
     <t>Composition.section.emptyReason</t>
   </si>
   <si>
-    <t>Empty reason</t>
+    <t>Raison pour laquelle la section est vide</t>
   </si>
   <si>
     <t>If the section is empty, why the list is empty. An empty section typically has some text explaining the empty reason.</t>
@@ -2775,7 +2778,7 @@
     <t>Composition.section.section</t>
   </si>
   <si>
-    <t>Nested Section</t>
+    <t>Sous-section</t>
   </si>
   <si>
     <t>A nested sub-section within this section.</t>
@@ -30663,7 +30666,7 @@
         <v>105</v>
       </c>
       <c r="L237" t="s" s="2">
-        <v>106</v>
+        <v>821</v>
       </c>
       <c r="M237" t="s" s="2">
         <v>107</v>
@@ -30749,10 +30752,10 @@
     </row>
     <row r="238" hidden="true">
       <c r="A238" t="s" s="2">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="B238" t="s" s="2">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C238" s="2"/>
       <c r="D238" t="s" s="2">
@@ -30862,13 +30865,13 @@
     </row>
     <row r="239" hidden="true">
       <c r="A239" t="s" s="2">
+        <v>823</v>
+      </c>
+      <c r="B239" t="s" s="2">
         <v>822</v>
       </c>
-      <c r="B239" t="s" s="2">
-        <v>821</v>
-      </c>
       <c r="C239" t="s" s="2">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="D239" t="s" s="2">
         <v>78</v>
@@ -30890,16 +30893,16 @@
         <v>78</v>
       </c>
       <c r="K239" t="s" s="2">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="L239" t="s" s="2">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="M239" t="s" s="2">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="N239" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="O239" s="2"/>
       <c r="P239" t="s" s="2">
@@ -30981,10 +30984,10 @@
     </row>
     <row r="240" hidden="true">
       <c r="A240" t="s" s="2">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="B240" t="s" s="2">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="C240" s="2"/>
       <c r="D240" t="s" s="2">
@@ -31100,14 +31103,14 @@
     </row>
     <row r="241">
       <c r="A241" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="C241" s="2"/>
       <c r="D241" t="s" s="2">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="E241" s="2"/>
       <c r="F241" t="s" s="2">
@@ -31129,16 +31132,16 @@
         <v>105</v>
       </c>
       <c r="L241" t="s" s="2">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="M241" t="s" s="2">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="N241" t="s" s="2">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="O241" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="P241" t="s" s="2">
         <v>78</v>
@@ -31187,7 +31190,7 @@
         <v>78</v>
       </c>
       <c r="AF241" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="AG241" t="s" s="2">
         <v>79</v>
@@ -31219,10 +31222,10 @@
     </row>
     <row r="242">
       <c r="A242" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="C242" s="2"/>
       <c r="D242" t="s" s="2">
@@ -31248,16 +31251,16 @@
         <v>276</v>
       </c>
       <c r="L242" t="s" s="2">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="M242" t="s" s="2">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="N242" t="s" s="2">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="O242" t="s" s="2">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="P242" t="s" s="2">
         <v>78</v>
@@ -31286,7 +31289,7 @@
       </c>
       <c r="Y242" s="2"/>
       <c r="Z242" t="s" s="2">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="AA242" t="s" s="2">
         <v>78</v>
@@ -31304,7 +31307,7 @@
         <v>78</v>
       </c>
       <c r="AF242" t="s" s="2">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="AG242" t="s" s="2">
         <v>79</v>
@@ -31336,10 +31339,10 @@
     </row>
     <row r="243" hidden="true">
       <c r="A243" t="s" s="2">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="B243" t="s" s="2">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="C243" s="2"/>
       <c r="D243" t="s" s="2">
@@ -31362,13 +31365,13 @@
         <v>78</v>
       </c>
       <c r="K243" t="s" s="2">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="L243" t="s" s="2">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="M243" t="s" s="2">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="N243" s="2"/>
       <c r="O243" t="s" s="2">
@@ -31421,7 +31424,7 @@
         <v>78</v>
       </c>
       <c r="AF243" t="s" s="2">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="AG243" t="s" s="2">
         <v>79</v>
@@ -31453,10 +31456,10 @@
     </row>
     <row r="244" hidden="true">
       <c r="A244" t="s" s="2">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="B244" t="s" s="2">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="C244" s="2"/>
       <c r="D244" t="s" s="2">
@@ -31482,13 +31485,13 @@
         <v>772</v>
       </c>
       <c r="L244" t="s" s="2">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="M244" t="s" s="2">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N244" t="s" s="2">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="O244" s="2"/>
       <c r="P244" t="s" s="2">
@@ -31538,7 +31541,7 @@
         <v>78</v>
       </c>
       <c r="AF244" t="s" s="2">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="AG244" t="s" s="2">
         <v>79</v>
@@ -31559,7 +31562,7 @@
         <v>78</v>
       </c>
       <c r="AM244" t="s" s="2">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="AN244" t="s" s="2">
         <v>78</v>
@@ -31570,10 +31573,10 @@
     </row>
     <row r="245">
       <c r="A245" t="s" s="2">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="B245" t="s" s="2">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C245" s="2"/>
       <c r="D245" t="s" s="2">
@@ -31599,13 +31602,13 @@
         <v>189</v>
       </c>
       <c r="L245" t="s" s="2">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="M245" t="s" s="2">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="N245" t="s" s="2">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="O245" s="2"/>
       <c r="P245" t="s" s="2">
@@ -31655,7 +31658,7 @@
         <v>78</v>
       </c>
       <c r="AF245" t="s" s="2">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="AG245" t="s" s="2">
         <v>79</v>
@@ -31664,7 +31667,7 @@
         <v>91</v>
       </c>
       <c r="AI245" t="s" s="2">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="AJ245" t="s" s="2">
         <v>103</v>
@@ -31673,10 +31676,10 @@
         <v>78</v>
       </c>
       <c r="AL245" t="s" s="2">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="AM245" t="s" s="2">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="AN245" t="s" s="2">
         <v>78</v>
@@ -31687,10 +31690,10 @@
     </row>
     <row r="246" hidden="true">
       <c r="A246" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B246" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="C246" s="2"/>
       <c r="D246" t="s" s="2">
@@ -31716,16 +31719,16 @@
         <v>179</v>
       </c>
       <c r="L246" t="s" s="2">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="M246" t="s" s="2">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="N246" t="s" s="2">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="O246" t="s" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="P246" t="s" s="2">
         <v>78</v>
@@ -31753,10 +31756,10 @@
         <v>358</v>
       </c>
       <c r="Y246" t="s" s="2">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="Z246" t="s" s="2">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="AA246" t="s" s="2">
         <v>78</v>
@@ -31774,7 +31777,7 @@
         <v>78</v>
       </c>
       <c r="AF246" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="AG246" t="s" s="2">
         <v>79</v>
@@ -31792,7 +31795,7 @@
         <v>78</v>
       </c>
       <c r="AL246" t="s" s="2">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="AM246" t="s" s="2">
         <v>109</v>
@@ -31806,10 +31809,10 @@
     </row>
     <row r="247" hidden="true">
       <c r="A247" t="s" s="2">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="B247" t="s" s="2">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="C247" s="2"/>
       <c r="D247" t="s" s="2">
@@ -31835,16 +31838,16 @@
         <v>276</v>
       </c>
       <c r="L247" t="s" s="2">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="M247" t="s" s="2">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="N247" t="s" s="2">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="O247" t="s" s="2">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="P247" t="s" s="2">
         <v>78</v>
@@ -31872,10 +31875,10 @@
         <v>183</v>
       </c>
       <c r="Y247" t="s" s="2">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="Z247" t="s" s="2">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="AA247" t="s" s="2">
         <v>78</v>
@@ -31893,7 +31896,7 @@
         <v>78</v>
       </c>
       <c r="AF247" t="s" s="2">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="AG247" t="s" s="2">
         <v>79</v>
@@ -31911,7 +31914,7 @@
         <v>78</v>
       </c>
       <c r="AL247" t="s" s="2">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="AM247" t="s" s="2">
         <v>109</v>
@@ -31925,10 +31928,10 @@
     </row>
     <row r="248" hidden="true">
       <c r="A248" t="s" s="2">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="B248" t="s" s="2">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C248" s="2"/>
       <c r="D248" t="s" s="2">
@@ -31954,13 +31957,13 @@
         <v>772</v>
       </c>
       <c r="L248" t="s" s="2">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="M248" t="s" s="2">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="N248" t="s" s="2">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="O248" s="2"/>
       <c r="P248" t="s" s="2">
@@ -32010,7 +32013,7 @@
         <v>78</v>
       </c>
       <c r="AF248" t="s" s="2">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="AG248" t="s" s="2">
         <v>79</v>
@@ -32019,7 +32022,7 @@
         <v>80</v>
       </c>
       <c r="AI248" t="s" s="2">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="AJ248" t="s" s="2">
         <v>103</v>
@@ -32028,10 +32031,10 @@
         <v>78</v>
       </c>
       <c r="AL248" t="s" s="2">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="AM248" t="s" s="2">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="AN248" t="s" s="2">
         <v>78</v>
@@ -32042,10 +32045,10 @@
     </row>
     <row r="249" hidden="true">
       <c r="A249" t="s" s="2">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B249" t="s" s="2">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="C249" s="2"/>
       <c r="D249" t="s" s="2">
@@ -32071,16 +32074,16 @@
         <v>276</v>
       </c>
       <c r="L249" t="s" s="2">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="M249" t="s" s="2">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="N249" t="s" s="2">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="O249" t="s" s="2">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="P249" t="s" s="2">
         <v>78</v>
@@ -32108,10 +32111,10 @@
         <v>183</v>
       </c>
       <c r="Y249" t="s" s="2">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="Z249" t="s" s="2">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="AA249" t="s" s="2">
         <v>78</v>
@@ -32129,7 +32132,7 @@
         <v>78</v>
       </c>
       <c r="AF249" t="s" s="2">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="AG249" t="s" s="2">
         <v>79</v>
@@ -32138,7 +32141,7 @@
         <v>91</v>
       </c>
       <c r="AI249" t="s" s="2">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="AJ249" t="s" s="2">
         <v>103</v>
@@ -32147,7 +32150,7 @@
         <v>78</v>
       </c>
       <c r="AL249" t="s" s="2">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="AM249" t="s" s="2">
         <v>109</v>
@@ -32161,10 +32164,10 @@
     </row>
     <row r="250" hidden="true">
       <c r="A250" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="B250" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C250" s="2"/>
       <c r="D250" t="s" s="2">
@@ -32190,13 +32193,13 @@
         <v>81</v>
       </c>
       <c r="L250" t="s" s="2">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="M250" t="s" s="2">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="N250" t="s" s="2">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="O250" s="2"/>
       <c r="P250" t="s" s="2">
@@ -32246,7 +32249,7 @@
         <v>78</v>
       </c>
       <c r="AF250" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="AG250" t="s" s="2">
         <v>79</v>
@@ -32255,7 +32258,7 @@
         <v>80</v>
       </c>
       <c r="AI250" t="s" s="2">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="AJ250" t="s" s="2">
         <v>103</v>
@@ -32267,7 +32270,7 @@
         <v>818</v>
       </c>
       <c r="AM250" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="AN250" t="s" s="2">
         <v>78</v>

</xml_diff>